<commit_message>
Daily EOD data and reports for 2026-08-20
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260820.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260820.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.702</v>
+        <v>1.72</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.107</v>
+        <v>0.125</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.71%</t>
+          <t>7.84%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>260714.06</v>
+        <v>263471.32</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>16390.37</v>
+        <v>19147.62</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.375</v>
+        <v>2.365</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.005</v>
+        <v>-0.015</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.21%</t>
+          <t>-0.63%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>166250</v>
+        <v>165550</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-350</v>
+        <v>-1050</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>65.16500000000001</v>
+        <v>65.22</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1.455</v>
+        <v>1.51</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.28%</t>
+          <t>2.37%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>721050.73</v>
+        <v>721659.3</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>16099.58</v>
+        <v>16708.15</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>158.83</v>
+        <v>156.89</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-1.88</v>
+        <v>-3.82</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>-2.38%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.96</v>
+        <v>0.962</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.09</v>
+        <v>0.092</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.34%</t>
+          <t>10.57%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9600</v>
+        <v>9620</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>900</v>
+        <v>920</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>171.01</v>
+        <v>173.62</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>4.53</v>
+        <v>7.14</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.72%</t>
+          <t>4.29%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>684040</v>
+        <v>694480</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>18120</v>
+        <v>28560</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.275</v>
+        <v>0.27</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3.77%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5500</v>
+        <v>5400</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.12</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>1129.44</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-1129.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.105</v>
+        <v>-0.005</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-630</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.07</v>
+        <v>33.74</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.37</v>
+        <v>-0.7</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>-2.03%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.45</v>
+        <v>33.56</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.1</v>
+        <v>0.01</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>0.03%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>43083.6</v>
+        <v>43225.28</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-128.8</v>
+        <v>12.88</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1890370.66</v>
+        <v>1905267.61</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-19154.16</v>
+        <v>-4257.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>